<commit_message>
switch to html version
</commit_message>
<xml_diff>
--- a/Data/Work History Summary.xlsx
+++ b/Data/Work History Summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paulb\R Projects\CV\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paulb\R\Projects\paul.beard.for.hire\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BAD829F-C240-400E-A2F9-3753C96A973B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB5B111F-A3BC-49F5-B7FF-E89546A8FB44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-15" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="19200" windowHeight="11170" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TeamsTasks" sheetId="1" r:id="rId1"/>
@@ -34,8 +34,26 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={AFD3B207-5223-4811-B274-A67714530234}</author>
+  </authors>
+  <commentList>
+    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{AFD3B207-5223-4811-B274-A67714530234}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Up to half-year</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="50">
   <si>
     <t>Team</t>
   </si>
@@ -140,9 +158,6 @@
   </si>
   <si>
     <t>Platform</t>
-  </si>
-  <si>
-    <t>Totes</t>
   </si>
   <si>
     <t>Excel</t>
@@ -271,6 +286,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Paul Beard" id="{CA7B08D5-C7C9-4C10-A16A-1C9083EB1D41}" userId="1d0d02321a030393" providerId="Windows Live"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -469,13 +490,21 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="M1" dT="2024-07-15T19:29:04.13" personId="{CA7B08D5-C7C9-4C10-A16A-1C9083EB1D41}" id="{AFD3B207-5223-4811-B274-A67714530234}">
+    <text>Up to half-year</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:F25"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="5" width="31" customWidth="1"/>
@@ -975,7 +1004,7 @@
         <v>33</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F25" s="1">
         <v>10</v>
@@ -987,14 +1016,14 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
@@ -1031,13 +1060,13 @@
       <c r="L1" s="1">
         <v>2023</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="1">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="B2" s="1">
         <v>1200</v>
@@ -1073,13 +1102,12 @@
         <v>1000</v>
       </c>
       <c r="M2" s="1">
-        <f t="shared" ref="M2:M7" si="0">SUM(B2:L2)</f>
-        <v>12000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="13.2" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B3" s="1">
         <v>0</v>
@@ -1115,13 +1143,12 @@
         <v>150</v>
       </c>
       <c r="M3" s="1">
-        <f t="shared" si="0"/>
-        <v>800</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="13.2" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B4" s="1">
         <v>125</v>
@@ -1157,13 +1184,12 @@
         <v>0</v>
       </c>
       <c r="M4" s="1">
-        <f>SUM(B4:L4)</f>
-        <v>625</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="13.2" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5" s="1">
         <v>0</v>
@@ -1190,22 +1216,21 @@
         <v>100</v>
       </c>
       <c r="J5" s="1">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="K5" s="1">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="L5" s="1">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="M5" s="1">
-        <f t="shared" si="0"/>
-        <v>1750</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="13.2" x14ac:dyDescent="0.25">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B6" s="1">
         <v>40</v>
@@ -1241,13 +1266,12 @@
         <v>0</v>
       </c>
       <c r="M6" s="1">
-        <f t="shared" si="0"/>
-        <v>160</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" s="1">
         <v>0</v>
@@ -1283,12 +1307,12 @@
         <v>50</v>
       </c>
       <c r="M7" s="1">
-        <f t="shared" si="0"/>
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1298,29 +1322,29 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -1334,7 +1358,7 @@
     </row>
     <row r="3" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B3">
         <v>0.09</v>
@@ -1348,7 +1372,7 @@
     </row>
     <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B4">
         <v>0.73</v>
@@ -1362,7 +1386,7 @@
     </row>
     <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B5">
         <v>0.94499999999999995</v>

</xml_diff>

<commit_message>
update spreadsheet of data
</commit_message>
<xml_diff>
--- a/Data/Work History Summary.xlsx
+++ b/Data/Work History Summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paulb\R\Projects\paul.beard.for.hire\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB5B111F-A3BC-49F5-B7FF-E89546A8FB44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A31A4B6A-0DA2-4FCB-ADC3-FF9491B32102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="19200" windowHeight="11170" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TeamsTasks" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="52">
   <si>
     <t>Team</t>
   </si>
@@ -203,6 +203,12 @@
   </si>
   <si>
     <t>count</t>
+  </si>
+  <si>
+    <t>Longevity Pricing</t>
+  </si>
+  <si>
+    <t>Model Migration to R</t>
   </si>
 </sst>
 </file>
@@ -503,7 +509,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1008,6 +1014,26 @@
       </c>
       <c r="F25" s="1">
         <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="2">
+        <v>45322</v>
+      </c>
+      <c r="C26" s="2">
+        <v>45657</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F26" s="1">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1102,7 +1128,7 @@
         <v>1000</v>
       </c>
       <c r="M2" s="1">
-        <v>200</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="12.5" x14ac:dyDescent="0.25">
@@ -1225,7 +1251,7 @@
         <v>400</v>
       </c>
       <c r="M5" s="1">
-        <v>700</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="12.5" x14ac:dyDescent="0.25">

</xml_diff>